<commit_message>
Update results spreadsheet for hybrid model analysis with new data
</commit_message>
<xml_diff>
--- a/cookie_model/Results_Paper_hybrid_keksfabrik_24h_multistarts_ipopt_new.xlsx
+++ b/cookie_model/Results_Paper_hybrid_keksfabrik_24h_multistarts_ipopt_new.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,82 +442,82 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1.449589967727661</v>
+        <v>8.310976505279541</v>
       </c>
       <c r="B2" t="n">
-        <v>1107.482141167329</v>
+        <v>2462.108151365816</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1.446709632873535</v>
+        <v>4.139544725418091</v>
       </c>
       <c r="B3" t="n">
-        <v>1091.369067286905</v>
+        <v>2421.232131700138</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1.647708892822266</v>
+        <v>4.818528652191162</v>
       </c>
       <c r="B4" t="n">
-        <v>1076.034822270599</v>
+        <v>2505.239389646709</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1.14326548576355</v>
+        <v>1.769354104995728</v>
       </c>
       <c r="B5" t="n">
-        <v>1106.470931787808</v>
+        <v>2452.943891758406</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1.654106855392456</v>
+        <v>2.264616727828979</v>
       </c>
       <c r="B6" t="n">
-        <v>1084.816045330476</v>
+        <v>2467.183797028139</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.8395950794219971</v>
+        <v>3.38422703742981</v>
       </c>
       <c r="B7" t="n">
-        <v>1070.647718934016</v>
+        <v>2448.943924547187</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1.251570701599121</v>
+        <v>4.40679407119751</v>
       </c>
       <c r="B8" t="n">
-        <v>1095.855838224289</v>
+        <v>2459.631516399929</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1.1354660987854</v>
+        <v>2.669427633285522</v>
       </c>
       <c r="B9" t="n">
-        <v>1069.981758645567</v>
+        <v>2452.904817078604</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.696880340576172</v>
+        <v>2.835189342498779</v>
       </c>
       <c r="B10" t="n">
-        <v>1118.995766110502</v>
+        <v>2427.761908372257</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.9418108463287354</v>
+        <v>2.98250675201416</v>
       </c>
       <c r="B11" t="n">
-        <v>1095.672502589936</v>
+        <v>2443.970136727457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>